<commit_message>
chore: update exercise import template with simplified examples
- Replaced template with cleaner version
- Simplified example questions to generic content (capital city, fruits)
- Uses proper newline-separated option format expected by import code
- Shortened instructions text
</commit_message>
<xml_diff>
--- a/angular/src/assets/习题导入模版.xlsx
+++ b/angular/src/assets/习题导入模版.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,37 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +63,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,91 +463,92 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="62" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>使用说明：
-1. 题目类型：单选题为1，多选题为2，填空题为3，问答题为4
-2. 选择题答案用数字表示：1=A, 2=B, 3=C, 4=D，多个答案用逗号分隔（支持中英文逗号）
-3. 填空题和问答题的答案为文本</t>
+1. 题目类型：单选题=1，多选题=2，填空=3，问答=4
+2. 选择题答案：1=A, 2=B, 3=C, 4=D，多个用逗号分隔
+3. 选择题选项请每行一个，不要写在同一行</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>题目内容</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>题目类型</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>答案</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>选择题选项</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>以下哪种线条最适合表现坚硬、锐利的物体质感（  ）</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" ht="70" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>中国的首都是以下哪个城市？</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>A. 曲线
-B. 虚线
-C. 粗实线
-D. 细实线</t>
+      <c r="C3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>A. 上海
+B. 北京
+C. 广州
+D. 深圳</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>以下哪些属于设计的三大构成部分（  ）</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" ht="70" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>以下哪些属于水果？（多选）</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1，2，3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>A. 平面构成
-B. 色彩构成
-C. 立体构成
-D. 空间构成</t>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1,3,4</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>A. 苹果
+B. 白菜
+C. 香蕉
+D. 葡萄</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(exercise): add QuestionAnalysis field, AI analysis, import template, fix multi-tenant delete
- Add QuestionAnalysis field to Exercise entity, DTOs, and Angular proxy models
- Merge AnswerExplanation into QuestionAnalysis (remove separate field from UI)
- Add AI analysis endpoint (POST /api/app/exercise/ai-analyze) using Qwen API
  - Auto-fills answer if missing, generates analysis combining knowledge points
    and answer explanation
- Update Excel import template with QuestionAnalysis column
- Fix ResolveExerciseHeader to parse QuestionAnalysis column
- Fix DeleteAsync/BatchRemoveAsync: add DataFilter.Disable<IMultiTenant>()
  to match GetByCourseAsync query scope (exercises visible but not deletable)
- Fix AiAnalysisResult JSON deserialization with JsonPropertyName attributes
- Fix system prompt passing to use ChatOptions.Instructions pattern
- Fix formatAnswer to show FillBlank/ShortAnswer text (first 10 chars)
</commit_message>
<xml_diff>
--- a/angular/src/assets/习题导入模版.xlsx
+++ b/angular/src/assets/习题导入模版.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +40,12 @@
       <name val="微软雅黑"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -55,7 +61,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -77,11 +83,17 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,6 +103,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -457,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -472,27 +487,33 @@
           <t>使用说明：
 1. 题目类型：单选题=1，多选题=2，填空=3，问答=4
 2. 选择题答案：1=A, 2=B, 3=C, 4=D，多个用逗号分隔
-3. 选择题选项请每行一个，不要写在同一行</t>
+3. 选择题选项请每行一个，不要写在同一行
+4. 题目解析（可选）：填写题目解析、解题思路、易错点提示等</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>题目内容</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>题目类型</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>答案</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>题目解析</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>选择题选项</t>
         </is>
@@ -510,7 +531,8 @@
       <c r="C3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>上海
 北京
@@ -533,7 +555,8 @@
           <t>1,3,4</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>苹果
 白菜
@@ -556,7 +579,8 @@
           <t>3×10⁸ m/s</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -572,7 +596,8 @@
           <t>答出叶绿体、光反应、暗反应即可</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>